<commit_message>
chore: update snitch default data and clean up old datasets
</commit_message>
<xml_diff>
--- a/defalut_data/snitch/snitch.xlsx
+++ b/defalut_data/snitch/snitch.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vivek kumar Gupta\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vivek kumar Gupta\Downloads\client-1-main\defalut_data\snitch\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{32A992F9-FEA5-402C-A82D-462879CB6F28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{95A3EDB8-3C62-4DA2-A812-4555F449CFE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3572,6 +3572,7 @@
     <col min="5" max="5" width="18.85546875" customWidth="1"/>
     <col min="6" max="6" width="12.5703125" customWidth="1"/>
     <col min="7" max="7" width="18.85546875" customWidth="1"/>
+    <col min="10" max="10" width="20.7109375" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.25">

</xml_diff>